<commit_message>
Make generated schedules vary within studio caps
</commit_message>
<xml_diff>
--- a/outputs/schedule_courtside.xlsx
+++ b/outputs/schedule_courtside.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,15 +43,20 @@
       <sz val="10"/>
     </font>
     <font>
+      <color rgb="006B21A8"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="10"/>
+    </font>
+    <font>
       <color rgb="000C4A6E"/>
       <sz val="9"/>
     </font>
-    <font>
-      <color rgb="006B21A8"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -75,12 +80,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D5F2F8"/>
+        <fgColor rgb="00E8D5FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8D5FF"/>
+        <fgColor rgb="00FFFBEB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F2F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -110,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -129,6 +139,9 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -496,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -568,7 +581,7 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="B3" s="5" t="n"/>
@@ -578,18 +591,18 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Mat 57
-Atulan Purohit
-20% pred | 0% hist
-[]</t>
+          <t>FIT
+Simran Dutt
+51% pred | 51% hist
+[INCLUDE]</t>
         </is>
       </c>
       <c r="H3" s="5" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>20:00</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>10:15</t>
         </is>
       </c>
       <c r="B4" s="5" t="n"/>
@@ -597,15 +610,57 @@
       <c r="D4" s="5" t="n"/>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57 Express
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Cardio Barre
+Karan Bhatia
+23% pred | 23% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Barre 57
+Anmol Sharma
+33% pred | 33% hist
+[INCLUDE]</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Mat 57
 Pranjali Jain
 20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="n"/>
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -621,7 +676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -693,7 +748,7 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="B3" s="5" t="n"/>
@@ -703,18 +758,18 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Mat 57
-Atulan Purohit
-20% pred | 0% hist
-[]</t>
+          <t>FIT
+Karan Bhatia
+51% pred | 51% hist
+[INCLUDE]</t>
         </is>
       </c>
       <c r="H3" s="5" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>20:00</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>10:15</t>
         </is>
       </c>
       <c r="B4" s="5" t="n"/>
@@ -722,15 +777,57 @@
       <c r="D4" s="5" t="n"/>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57 Express
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Barre 57
+Karan Bhatia
+47% pred | 47% hist
+[INCLUDE]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Barre 57
+Anmol Sharma
+33% pred | 33% hist
+[INCLUDE]</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Mat 57
 Pranjali Jain
 20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="n"/>
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -746,7 +843,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -818,7 +915,7 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="B3" s="5" t="n"/>
@@ -828,18 +925,18 @@
       <c r="F3" s="5" t="n"/>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Mat 57
-Atulan Purohit
-20% pred | 0% hist
-[]</t>
+          <t>FIT
+Simran Dutt
+51% pred | 51% hist
+[INCLUDE]</t>
         </is>
       </c>
       <c r="H3" s="5" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>20:00</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>10:15</t>
         </is>
       </c>
       <c r="B4" s="5" t="n"/>
@@ -847,15 +944,57 @@
       <c r="D4" s="5" t="n"/>
       <c r="E4" s="5" t="n"/>
       <c r="F4" s="5" t="n"/>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Barre 57 Express
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>Cardio Barre
+Karan Bhatia
+23% pred | 23% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Barre 57
+Anmol Sharma
+33% pred | 33% hist
+[INCLUDE]</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Mat 57
 Pranjali Jain
 20% pred | 0% hist
-[]</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="n"/>
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>